<commit_message>
Dashboard de precios terminado
</commit_message>
<xml_diff>
--- a/Ejercicios_Estadistica_Alumnos.xlsx
+++ b/Ejercicios_Estadistica_Alumnos.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Proyectos/cursos_activos/inserta_once/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Proyectos/cursos_activos/inserta_once/big_data/materias/matematicas/analisis_estadistico/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54222956-CA8B-9540-87B0-F23EEB278FBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86FE22DD-078E-B54C-B355-4C3FBE22A13F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="140" yWindow="740" windowWidth="38080" windowHeight="19940" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18220" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos_Base" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,12 @@
     <sheet name="3_Satisfaccion" sheetId="4" r:id="rId4"/>
     <sheet name="4_Probabilidad" sheetId="5" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">'1_Precios'!$A$5:$A$46</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">'1_Precios'!$B$5:$B$46</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">'1_Precios'!$A$5:$A$46</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">'1_Precios'!$B$5:$B$46</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -37,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="153">
   <si>
     <t>ID_Venta</t>
   </si>
@@ -487,6 +493,15 @@
   </si>
   <si>
     <t>Dashboard 4: Probabilidad y Frecuencias (Canales)</t>
+  </si>
+  <si>
+    <t>18 es el producto que mas se ha comprado</t>
+  </si>
+  <si>
+    <t>media y mediana no son parececidas, esto implica mucho outliners, valores extremos sobre todo todo en la parte alta que distorsionan la media</t>
+  </si>
+  <si>
+    <t>el ticket medio de nuestra tienda es 35</t>
   </si>
 </sst>
 </file>
@@ -574,7 +589,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -597,6 +612,19 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -608,16 +636,66 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -628,6 +706,724 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
+<cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
+  <cx:chartData>
+    <cx:data id="0">
+      <cx:strDim type="cat">
+        <cx:f>_xlchart.v1.0</cx:f>
+      </cx:strDim>
+      <cx:numDim type="val">
+        <cx:f>_xlchart.v1.1</cx:f>
+      </cx:numDim>
+    </cx:data>
+  </cx:chartData>
+  <cx:chart>
+    <cx:title pos="t" align="ctr" overlay="0">
+      <cx:tx>
+        <cx:txData>
+          <cx:v>Histograma de precios</cx:v>
+        </cx:txData>
+      </cx:tx>
+      <cx:txPr>
+        <a:bodyPr spcFirstLastPara="1" vertOverflow="ellipsis" horzOverflow="overflow" wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr" rtl="0">
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="es-ES" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:sysClr>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:rPr>
+            <a:t>Histograma de precios</a:t>
+          </a:r>
+        </a:p>
+      </cx:txPr>
+    </cx:title>
+    <cx:plotArea>
+      <cx:plotAreaRegion>
+        <cx:series layoutId="clusteredColumn" uniqueId="{949CBF06-2D9B-FB48-96BF-095B9EE0F8CE}">
+          <cx:dataId val="0"/>
+          <cx:layoutPr>
+            <cx:binning intervalClosed="r"/>
+          </cx:layoutPr>
+        </cx:series>
+      </cx:plotAreaRegion>
+      <cx:axis id="0">
+        <cx:catScaling gapWidth="0"/>
+        <cx:tickLabels/>
+      </cx:axis>
+      <cx:axis id="1">
+        <cx:valScaling/>
+        <cx:majorGridlines/>
+        <cx:tickLabels/>
+      </cx:axis>
+    </cx:plotArea>
+  </cx:chart>
+</cx:chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="phClr"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat">
+        <a:solidFill>
+          <a:srgbClr val="D9D9D9"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDash"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>2056</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>14088</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>460696</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>93887</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" Requires="cx1">
+        <xdr:graphicFrame macro="">
+          <xdr:nvGraphicFramePr>
+            <xdr:cNvPr id="2" name="Gráfico 1">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{35692A52-AF2D-E096-9BEC-0C1945AEFBAB}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvGraphicFramePr/>
+          </xdr:nvGraphicFramePr>
+          <xdr:xfrm>
+            <a:off x="0" y="0"/>
+            <a:ext cx="0" cy="0"/>
+          </xdr:xfrm>
+          <a:graphic>
+            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2014/chartex">
+              <cx:chart xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+            </a:graphicData>
+          </a:graphic>
+        </xdr:graphicFrame>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="0" name=""/>
+            <xdr:cNvSpPr>
+              <a:spLocks noTextEdit="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4722137" y="2158177"/>
+              <a:ext cx="4572000" cy="2743200"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:solidFill>
+              <a:prstClr val="white"/>
+            </a:solidFill>
+            <a:ln w="1">
+              <a:solidFill>
+                <a:prstClr val="green"/>
+              </a:solidFill>
+            </a:ln>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:r>
+                <a:rPr lang="es-ES_tradnl" sz="1100"/>
+                <a:t>Este gráfico no está disponible en su versión de Excel.
+Si edita esta forma o guarda el libro en un formato de archivo diferente, el gráfico no se podrá utilizar.</a:t>
+              </a:r>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E676DA87-2E3F-E746-8DEB-EBB0A3A138E2}" name="Tabla1" displayName="Tabla1" ref="A1:N43" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="1" tableBorderDxfId="2">
+  <autoFilter ref="A1:N43" xr:uid="{E676DA87-2E3F-E746-8DEB-EBB0A3A138E2}"/>
+  <tableColumns count="14">
+    <tableColumn id="1" xr3:uid="{26D470CC-E5AA-4348-9460-96D5EFC4DB1E}" name="ID_Venta"/>
+    <tableColumn id="2" xr3:uid="{FE993127-7F97-BD41-953F-77B8033BD5D1}" name="Fecha"/>
+    <tableColumn id="3" xr3:uid="{673C1234-03BF-244D-8281-83FA862CBA6C}" name="Producto"/>
+    <tableColumn id="4" xr3:uid="{CE5BEC10-5201-904E-95DB-1E6142DB006F}" name="Categoría"/>
+    <tableColumn id="5" xr3:uid="{9A849799-0BF3-6846-A1D5-41987B4C96D3}" name="Unidades"/>
+    <tableColumn id="6" xr3:uid="{F45D335E-10A1-084C-8EB7-C3F28E54C1AD}" name="Precio_Unitario"/>
+    <tableColumn id="7" xr3:uid="{107591FF-B401-464B-981D-EEAAA9529E4B}" name="Ciudad"/>
+    <tableColumn id="8" xr3:uid="{47F38C4D-F1F5-C04A-B40E-4D25E11D90C2}" name="Canal"/>
+    <tableColumn id="9" xr3:uid="{04A571EB-F1E1-BF4F-9CF2-44A128B37E11}" name="Valoración"/>
+    <tableColumn id="10" xr3:uid="{B1A0E6CA-3F1D-744D-802F-BB647FC7F717}" name="Ingresos"/>
+    <tableColumn id="11" xr3:uid="{D5F2F345-DA4B-7140-9BB1-542587C7B105}" name="Coste"/>
+    <tableColumn id="12" xr3:uid="{7B44BF3E-72B4-F94C-B893-06D468B4A133}" name="Beneficio"/>
+    <tableColumn id="13" xr3:uid="{40370B9E-7AEC-FC40-994E-15F17556796D}" name="Vendedor"/>
+    <tableColumn id="14" xr3:uid="{4779B0E5-D868-3544-A152-CBE33F5DD4B1}" name="Devolución"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -919,48 +1715,60 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="10.6640625" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" customWidth="1"/>
+    <col min="6" max="6" width="15.6640625" customWidth="1"/>
+    <col min="9" max="9" width="11.83203125" customWidth="1"/>
+    <col min="10" max="10" width="9.83203125" customWidth="1"/>
+    <col min="12" max="12" width="10.83203125" customWidth="1"/>
+    <col min="13" max="13" width="11.33203125" customWidth="1"/>
+    <col min="14" max="14" width="12.33203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="M1" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="N1" s="8" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2814,6 +3622,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -2857,7 +3668,10 @@
       <c r="D5" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="E5" s="4"/>
+      <c r="E5" s="4">
+        <f>AVERAGE(B5:B46)</f>
+        <v>60.011904761904759</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
@@ -2869,7 +3683,10 @@
       <c r="D6" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="E6" s="4"/>
+      <c r="E6" s="4">
+        <f>MEDIAN(B5:B46)</f>
+        <v>35</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -2881,7 +3698,10 @@
       <c r="D7" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="E7" s="4"/>
+      <c r="E7" s="4">
+        <f>_xlfn.MODE.SNGL(B5:B46)</f>
+        <v>18</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -2893,7 +3713,10 @@
       <c r="D8" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="E8" s="4"/>
+      <c r="E8" s="4">
+        <f>_xlfn.STDEV.S(B5:B46)</f>
+        <v>63.23692269082472</v>
+      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -2962,7 +3785,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>68</v>
       </c>
@@ -2970,7 +3793,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>69</v>
       </c>
@@ -2978,7 +3801,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>70</v>
       </c>
@@ -2986,7 +3809,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>71</v>
       </c>
@@ -2994,7 +3817,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>72</v>
       </c>
@@ -3002,7 +3825,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>73</v>
       </c>
@@ -3010,7 +3833,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>74</v>
       </c>
@@ -3018,7 +3841,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>75</v>
       </c>
@@ -3026,7 +3849,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>76</v>
       </c>
@@ -3034,7 +3857,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>77</v>
       </c>
@@ -3042,7 +3865,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>78</v>
       </c>
@@ -3050,7 +3873,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>79</v>
       </c>
@@ -3058,31 +3881,40 @@
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>80</v>
       </c>
       <c r="B29">
         <v>120</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D29" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>81</v>
       </c>
       <c r="B30">
         <v>6</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D30" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>82</v>
       </c>
       <c r="B31">
         <v>12</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="D31" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>83</v>
       </c>
@@ -3204,6 +4036,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4201,8 +5034,8 @@
         <v>110</v>
       </c>
       <c r="E6" s="4"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="7"/>
+      <c r="F6" s="7"/>
+      <c r="G6" s="6"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -4215,8 +5048,8 @@
         <v>111</v>
       </c>
       <c r="E7" s="4"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="7"/>
+      <c r="F7" s="7"/>
+      <c r="G7" s="6"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -4229,8 +5062,8 @@
         <v>112</v>
       </c>
       <c r="E8" s="4"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="7"/>
+      <c r="F8" s="7"/>
+      <c r="G8" s="6"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -4243,8 +5076,8 @@
         <v>143</v>
       </c>
       <c r="E9" s="4"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="6"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">

</xml_diff>

<commit_message>
Valoracion de satisfacción terminada.
</commit_message>
<xml_diff>
--- a/Ejercicios_Estadistica_Alumnos.xlsx
+++ b/Ejercicios_Estadistica_Alumnos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Proyectos/cursos_activos/inserta_once/big_data/materias/matematicas/analisis_estadistico/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCDD09A7-8380-204E-9001-347EA8EB88AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D75F1732-6FB5-204D-BF30-1F4069D687DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18220" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20" yWindow="660" windowWidth="30240" windowHeight="18220" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos_Base" sheetId="1" r:id="rId1"/>
@@ -22,8 +22,6 @@
   <definedNames>
     <definedName name="_xlchart.v1.0" hidden="1">'1_Precios'!$A$5:$A$46</definedName>
     <definedName name="_xlchart.v1.1" hidden="1">'1_Precios'!$B$5:$B$46</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">'1_Precios'!$A$5:$A$46</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">'1_Precios'!$B$5:$B$46</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -647,6 +645,20 @@
   </cellStyles>
   <dxfs count="3">
     <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <i val="0"/>
@@ -679,20 +691,6 @@
         </right>
         <top/>
         <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color auto="1"/>
-        </top>
       </border>
     </dxf>
   </dxfs>
@@ -1282,6 +1280,316 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES_tradnl"/>
+              <a:t>Distribucción de Satisfacción</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent3">
+                <a:lumMod val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>'3_Satisfaccion'!$D$12:$D$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'3_Satisfaccion'!$E$12:$E$16</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>16</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-4EE3-0F4D-8B24-1E8058214E12}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="26"/>
+        <c:overlap val="17"/>
+        <c:axId val="524661440"/>
+        <c:axId val="524649792"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="524661440"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="524649792"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="524649792"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-ES"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="524661440"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-ES"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
 <cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
   <cx:chartData>
@@ -1426,6 +1734,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
   <cs:axisTitle>
@@ -2431,6 +2779,509 @@
         <a:round/>
       </a:ln>
     </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:valueAxis>
   <cs:wall>
@@ -2499,8 +3350,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="4722137" y="2158177"/>
-              <a:ext cx="4572000" cy="2743200"/>
+              <a:off x="4726456" y="2160388"/>
+              <a:ext cx="4573440" cy="2746799"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -2574,8 +3425,49 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1173386</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>11375</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>447226</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>136661</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Gráfico 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{25715B2D-046B-49FE-0BCF-03A7C1BA551A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E676DA87-2E3F-E746-8DEB-EBB0A3A138E2}" name="Tabla1" displayName="Tabla1" ref="A1:N43" totalsRowShown="0" headerRowDxfId="0" headerRowBorderDxfId="1" tableBorderDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E676DA87-2E3F-E746-8DEB-EBB0A3A138E2}" name="Tabla1" displayName="Tabla1" ref="A1:N43" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1" tableBorderDxfId="0">
   <autoFilter ref="A1:N43" xr:uid="{E676DA87-2E3F-E746-8DEB-EBB0A3A138E2}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{26D470CC-E5AA-4348-9460-96D5EFC4DB1E}" name="ID_Venta"/>
@@ -5783,7 +6675,10 @@
       <c r="D5" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="E5" s="4"/>
+      <c r="E5" s="4">
+        <f>AVERAGE(B5:B46)</f>
+        <v>4.2857142857142856</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
@@ -5795,7 +6690,10 @@
       <c r="D6" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="E6" s="4"/>
+      <c r="E6" s="4">
+        <f>MEDIAN(B5:B46)</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -5807,7 +6705,10 @@
       <c r="D7" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="E7" s="4"/>
+      <c r="E7" s="4">
+        <f>_xlfn.MODE.SNGL(B5:B46)</f>
+        <v>4</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -5860,7 +6761,10 @@
       <c r="D12" s="3">
         <v>1</v>
       </c>
-      <c r="E12" s="4"/>
+      <c r="E12" s="4">
+        <f>COUNTIF(B5:B46,D12)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
@@ -5872,7 +6776,10 @@
       <c r="D13" s="3">
         <v>2</v>
       </c>
-      <c r="E13" s="4"/>
+      <c r="E13" s="4">
+        <f t="shared" ref="E13:E16" si="0">COUNTIF(B6:B47,D13)</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -5884,7 +6791,10 @@
       <c r="D14" s="3">
         <v>3</v>
       </c>
-      <c r="E14" s="4"/>
+      <c r="E14" s="4">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -5896,7 +6806,10 @@
       <c r="D15" s="3">
         <v>4</v>
       </c>
-      <c r="E15" s="4"/>
+      <c r="E15" s="4">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -5908,7 +6821,10 @@
       <c r="D16" s="3">
         <v>5</v>
       </c>
-      <c r="E16" s="4"/>
+      <c r="E16" s="4">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
@@ -6155,6 +7071,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Tabla de probabilidad terminada
</commit_message>
<xml_diff>
--- a/Ejercicios_Estadistica_Alumnos.xlsx
+++ b/Ejercicios_Estadistica_Alumnos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Proyectos/cursos_activos/inserta_once/big_data/materias/matematicas/analisis_estadistico/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D75F1732-6FB5-204D-BF30-1F4069D687DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8512908E-4487-1D40-B8B5-182874257AA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="660" windowWidth="30240" windowHeight="18220" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos_Base" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,8 @@
   <definedNames>
     <definedName name="_xlchart.v1.0" hidden="1">'1_Precios'!$A$5:$A$46</definedName>
     <definedName name="_xlchart.v1.1" hidden="1">'1_Precios'!$B$5:$B$46</definedName>
+    <definedName name="_xlchart.v1.2" hidden="1">'4_Probabilidad'!$D$6:$D$8</definedName>
+    <definedName name="_xlchart.v1.3" hidden="1">'4_Probabilidad'!$E$6:$E$8</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="572" uniqueCount="154">
   <si>
     <t>ID_Venta</t>
   </si>
@@ -500,6 +502,9 @@
   </si>
   <si>
     <t>el ticket medio de nuestra tienda es 35</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -1590,6 +1595,337 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-ES_tradnl"/>
+              <a:t>Probabilidad /Ventas por canal</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:view3D>
+      <c:rotX val="50"/>
+      <c:hPercent val="100"/>
+      <c:rotY val="0"/>
+      <c:depthPercent val="100"/>
+      <c:rAngAx val="0"/>
+      <c:perspective val="0"/>
+    </c:view3D>
+    <c:floor>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:floor>
+    <c:sideWall>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:sideWall>
+    <c:backWall>
+      <c:thickness val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+        <a:sp3d/>
+      </c:spPr>
+    </c:backWall>
+    <c:plotArea>
+      <c:layout/>
+      <c:pie3DChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="25400">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+              <a:scene3d>
+                <a:camera prst="orthographicFront"/>
+                <a:lightRig rig="threePt" dir="t"/>
+              </a:scene3d>
+              <a:sp3d contourW="25400" prstMaterial="metal">
+                <a:contourClr>
+                  <a:schemeClr val="lt1"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-8C78-4E4F-8B58-A5B59688176D}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="25400">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d contourW="25400">
+                <a:contourClr>
+                  <a:schemeClr val="lt1"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000002-8C78-4E4F-8B58-A5B59688176D}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="25400">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+              <a:sp3d contourW="25400">
+                <a:contourClr>
+                  <a:schemeClr val="lt1"/>
+                </a:contourClr>
+              </a:sp3d>
+            </c:spPr>
+          </c:dPt>
+          <c:cat>
+            <c:strRef>
+              <c:f>'4_Probabilidad'!$D$6:$D$8</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>App</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Web</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Tienda</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'4_Probabilidad'!$E$6:$E$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>14</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-8C78-4E4F-8B58-A5B59688176D}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+      </c:pie3DChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-ES"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+    <a:scene3d>
+      <a:camera prst="orthographicFront"/>
+      <a:lightRig rig="threePt" dir="t"/>
+    </a:scene3d>
+    <a:sp3d prstMaterial="dkEdge"/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-ES"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/chartEx1.xml><?xml version="1.0" encoding="utf-8"?>
 <cx:chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex">
   <cx:chartData>
@@ -1774,6 +2110,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="366">
   <cs:axisTitle>
@@ -3269,6 +3645,525 @@
             <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:upBar>
@@ -3446,6 +4341,47 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{25715B2D-046B-49FE-0BCF-03A7C1BA551A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>8589</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>189825</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>230686</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>80126</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="4" name="Gráfico 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2A38E43A-68D3-F54C-41C4-FD3381208CE6}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -7094,7 +8030,10 @@
       <c r="D3" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="E3" s="4"/>
+      <c r="E3" s="4">
+        <f>COUNTA(A5:A46)</f>
+        <v>42</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
@@ -7134,9 +8073,18 @@
       <c r="D6" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="E6" s="4"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="6"/>
+      <c r="E6" s="4">
+        <f>COUNTIF($B$5:$B$46,D6)</f>
+        <v>11</v>
+      </c>
+      <c r="F6" s="7">
+        <f>E6/$E$3</f>
+        <v>0.26190476190476192</v>
+      </c>
+      <c r="G6" s="6">
+        <f>F6</f>
+        <v>0.26190476190476192</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -7148,9 +8096,18 @@
       <c r="D7" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="E7" s="4"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="6"/>
+      <c r="E7" s="4">
+        <f>COUNTIF($B$5:$B$46,D7)</f>
+        <v>17</v>
+      </c>
+      <c r="F7" s="7">
+        <f t="shared" ref="F7:F8" si="0">E7/$E$3</f>
+        <v>0.40476190476190477</v>
+      </c>
+      <c r="G7" s="6">
+        <f t="shared" ref="G7:G8" si="1">F7</f>
+        <v>0.40476190476190477</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -7162,9 +8119,18 @@
       <c r="D8" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="E8" s="4"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="6"/>
+      <c r="E8" s="4">
+        <f>COUNTIF($B$5:$B$46,D8)</f>
+        <v>14</v>
+      </c>
+      <c r="F8" s="7">
+        <f t="shared" si="0"/>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="G8" s="6">
+        <f t="shared" si="1"/>
+        <v>0.33333333333333331</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -7176,9 +8142,18 @@
       <c r="D9" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="E9" s="4"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="6"/>
+      <c r="E9" s="4">
+        <f>SUM(E6:E8)</f>
+        <v>42</v>
+      </c>
+      <c r="F9" s="7">
+        <f>SUM(F6:F8)</f>
+        <v>1</v>
+      </c>
+      <c r="G9" s="6">
+        <f>F9</f>
+        <v>1</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
@@ -7248,7 +8223,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>68</v>
       </c>
@@ -7259,7 +8234,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>69</v>
       </c>
@@ -7267,7 +8242,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>70</v>
       </c>
@@ -7275,7 +8250,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>71</v>
       </c>
@@ -7283,7 +8258,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>72</v>
       </c>
@@ -7291,15 +8266,18 @@
         <v>112</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>73</v>
       </c>
       <c r="B22" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="G22" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>74</v>
       </c>
@@ -7307,7 +8285,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>75</v>
       </c>
@@ -7315,7 +8293,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>76</v>
       </c>
@@ -7323,7 +8301,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>77</v>
       </c>
@@ -7331,7 +8309,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>78</v>
       </c>
@@ -7339,7 +8317,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>79</v>
       </c>
@@ -7347,7 +8325,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>80</v>
       </c>
@@ -7355,7 +8333,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>81</v>
       </c>
@@ -7363,7 +8341,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>82</v>
       </c>
@@ -7371,7 +8349,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>83</v>
       </c>
@@ -7493,5 +8471,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>